<commit_message>
all products v1 completed
</commit_message>
<xml_diff>
--- a/src/reference_xls/inventory_xl.xlsx
+++ b/src/reference_xls/inventory_xl.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snigdhagoel/Documents/Vibrant Technik/vibrant-technik/material-calculator/reference_xls/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snigdhagoel/Documents/Vibrant Technik/vibrant-technik/tabular-entry/src/reference_xls/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D50F75A-FE30-6C46-8243-67E81247BA07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4F389D6-C7CB-E347-AA2A-C85EA99A5BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15940" xr2:uid="{6B53A8BC-CEAD-3D41-BD1D-F4619317B36C}"/>
   </bookViews>
@@ -673,7 +673,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -702,7 +702,13 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -710,8 +716,9 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -823,7 +830,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -834,14 +841,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -849,9 +853,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1224,32 +1225,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="8"/>
-      <c r="B1" s="8"/>
-      <c r="C1" s="9" t="s">
+      <c r="A1" s="7"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="14"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="12"/>
     </row>
     <row r="2" spans="1:11" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="17"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="15"/>
     </row>
     <row r="3" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1282,789 +1283,571 @@
       <c r="J3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="K3" s="1" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B4" s="6"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7">
+      <c r="E4" s="5">
         <f>D4</f>
         <v>0</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="5">
         <f t="shared" ref="F4:F35" si="0">IF(ISBLANK(C4), E4,ROUND(((C4*E4)/1000), 2))</f>
         <v>0</v>
       </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B5" s="6"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7">
+      <c r="E5" s="5">
         <f t="shared" ref="E5:E55" si="1">D5</f>
         <v>0</v>
       </c>
-      <c r="F5" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
+      <c r="F5" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B6" s="6"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F6" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
+      <c r="E6" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B7" s="6"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F7" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
+      <c r="E7" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F7" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B8" s="6"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F8" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+      <c r="E8" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F8" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B9" s="6"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F9" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
+      <c r="E9" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F9" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B10" s="6"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F10" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
+      <c r="E10" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F10" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B11" s="6"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F11" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
+      <c r="E11" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F11" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B12" s="6"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F12" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
+      <c r="E12" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F12" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B13" s="6"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F13" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
+      <c r="E13" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F13" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B14" s="6"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F14" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
+      <c r="E14" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F14" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B15" s="6"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F15" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
+      <c r="E15" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F15" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B16" s="6"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F16" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E16" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F16" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B17" s="6"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F17" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E17" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F17" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B18" s="6"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F18" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E18" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F18" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B19" s="6"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F19" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E19" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F19" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B20" s="6"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F20" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E20" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B21" s="6"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F21" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E21" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F21" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22" s="6"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F22" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E22" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F22" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B23" s="6"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F23" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E23" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F23" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B24" s="6"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F24" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E24" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F24" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B25" s="6"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F25" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E25" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F25" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B26" s="6"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F26" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E26" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F26" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B27" s="6"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F27" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E27" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F27" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B28" s="6"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F28" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-    </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E28" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F28" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B29" s="6"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F29" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E29" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F29" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30" s="6"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F30" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G30" s="7"/>
-      <c r="H30" s="7"/>
-    </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E30" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F30" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B31" s="6"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F31" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-    </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E31" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F31" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B32" s="6"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F32" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E32" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F32" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B33" s="6"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F33" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-    </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E33" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F33" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B34" s="6"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F34" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G34" s="7"/>
-      <c r="H34" s="7"/>
-    </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E34" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F34" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B35" s="6"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F35" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G35" s="7"/>
-      <c r="H35" s="7"/>
-    </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E35" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F35" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B36" s="6"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F36" s="7">
-        <f t="shared" ref="F36:F67" si="2">IF(ISBLANK(C36), E36,ROUND(((C36*E36)/1000), 2))</f>
-        <v>0</v>
-      </c>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-    </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="E36" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F36" s="5">
+        <f t="shared" ref="F36:F55" si="2">IF(ISBLANK(C36), E36,ROUND(((C36*E36)/1000), 2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B37" s="6"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F37" s="7">
+      <c r="E37" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F37" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38" s="6"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F38" s="7">
+      <c r="E38" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F38" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B39" s="6"/>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F39" s="7">
+      <c r="E39" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F39" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G39" s="7"/>
-      <c r="H39" s="7"/>
-    </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B40" s="6"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F40" s="7">
+      <c r="E40" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F40" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G40" s="7"/>
-      <c r="H40" s="7"/>
-    </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B41" s="6"/>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F41" s="7">
+      <c r="E41" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F41" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G41" s="7"/>
-      <c r="H41" s="7"/>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B42" s="6"/>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F42" s="7">
+      <c r="E42" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F42" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G42" s="7"/>
-      <c r="H42" s="7"/>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B43" s="6"/>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F43" s="7">
+      <c r="E43" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F43" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G43" s="7"/>
-      <c r="H43" s="7"/>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B44" s="6"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F44" s="7">
+      <c r="E44" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F44" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G44" s="7"/>
-      <c r="H44" s="7"/>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B45" s="6"/>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F45" s="7">
+      <c r="E45" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F45" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G45" s="7"/>
-      <c r="H45" s="7"/>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F46" s="7">
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="E46" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F46" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G46" s="7"/>
-      <c r="H46" s="7"/>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F47" s="7">
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="E47" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F47" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G47" s="7"/>
-      <c r="H47" s="7"/>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B48" s="7"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
-      <c r="E48" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F48" s="7">
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="E48" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F48" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G48" s="7"/>
-      <c r="H48" s="7"/>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B49" s="7"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
-      <c r="E49" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F49" s="7">
+    </row>
+    <row r="49" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E49" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F49" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G49" s="7"/>
-      <c r="H49" s="7"/>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F50" s="7">
+    </row>
+    <row r="50" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E50" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F50" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G50" s="7"/>
-      <c r="H50" s="7"/>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B51" s="7"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F51" s="7">
+    </row>
+    <row r="51" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E51" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F51" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G51" s="7"/>
-      <c r="H51" s="7"/>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B52" s="7"/>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
-      <c r="E52" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F52" s="7">
+    </row>
+    <row r="52" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E52" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F52" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G52" s="7"/>
-      <c r="H52" s="7"/>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
-      <c r="E53" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F53" s="7">
+    </row>
+    <row r="53" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E53" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F53" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G53" s="7"/>
-      <c r="H53" s="7"/>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B54" s="7"/>
-      <c r="C54" s="7"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F54" s="7">
+    </row>
+    <row r="54" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E54" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F54" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G54" s="7"/>
-      <c r="H54" s="7"/>
-    </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B55" s="7"/>
-      <c r="C55" s="7"/>
-      <c r="D55" s="7"/>
-      <c r="E55" s="7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F55" s="7">
+    </row>
+    <row r="55" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E55" s="5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F55" s="5">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G55" s="7"/>
-      <c r="H55" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>